<commit_message>
Clarify the evaluation spreadsheet criteria
Replace abbreviated criterion headers with descriptive titles so evaluators can identify each scoring category directly in the worksheet.

👾 Generated with [Letta Code](https://letta.com)

Co-Authored-By: Letta Code <noreply@letta.com>
</commit_message>
<xml_diff>
--- a/evaluacion/plantilla_evaluacion_proyectos.xlsx
+++ b/evaluacion/plantilla_evaluacion_proyectos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="83">
   <si>
     <t xml:space="preserve">Evaluaciones comunes — tres entregas / cinco grupos</t>
   </si>
@@ -47,139 +47,160 @@
     <t xml:space="preserve">Repositorio / PR</t>
   </si>
   <si>
+    <t xml:space="preserve">C1 — Especificación y restricciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 — Modelo y arquitectura del sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3 — Implementación técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4 — Integración hardware-software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5 — Verificación, pruebas y depuración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C6 — Integración y funcionamiento del sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7 — Documentación y sustentación técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos equipo / 90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidencia revisada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C8 individual — cinco espacios por grupo y evaluación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estudiante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable / usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issue / PR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C8 — Planificación, GitHub y responsabilidad individual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos C8 / 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota total / 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen de evaluaciones por grupo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación 1 / 90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación 2 / 90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación 3 / 90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promedio / 90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observaciones generales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota final por estudiante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos comunes del equipo (máx. 90) + C8 individual (máx. 10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rúbrica de evaluación de proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripción</t>
+  </si>
+  <si>
     <t xml:space="preserve">C1</t>
   </si>
   <si>
+    <t xml:space="preserve">Especificación y restricciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Función, interfaces, restricciones y criterios de aceptación.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C2</t>
   </si>
   <si>
+    <t xml:space="preserve">Modelo y arquitectura del sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloques, datapath, control, buses y decisiones justificadas.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C3</t>
   </si>
   <si>
+    <t xml:space="preserve">Implementación técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulos correctos, sintetizables e integrables.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C4</t>
   </si>
   <si>
+    <t xml:space="preserve">Integración hardware-software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firmware, mapa de memoria, CSR y control verificable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C5</t>
   </si>
   <si>
+    <t xml:space="preserve">Verificación, pruebas y depuración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pruebas reproducibles y análisis de resultados.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C6</t>
   </si>
   <si>
+    <t xml:space="preserve">Integración y funcionamiento del sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operación en la plataforma objetivo dentro del sistema.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puntos equipo / 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidencia revisada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observaciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C8 individual — cinco espacios por grupo y evaluación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estudiante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Responsable / usuario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Issue / PR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nivel C8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puntos C8 / 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nota total / 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumen de evaluaciones por grupo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluación 1 / 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluación 2 / 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluación 3 / 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Promedio / 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observaciones generales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nota final por estudiante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puntos comunes del equipo (máx. 90) + C8 individual (máx. 10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rúbrica de evaluación de proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descripción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Especificación y restricciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Función, interfaces, restricciones y criterios de aceptación.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo y arquitectura del sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloques, datapath, control, buses y decisiones justificadas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementación técnica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Módulos correctos, sintetizables e integrables.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integración hardware-software</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firmware, mapa de memoria, CSR y control verificable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificación, pruebas y depuración</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pruebas reproducibles y análisis de resultados.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integración y funcionamiento del sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operación en la plataforma objetivo dentro del sistema.</t>
   </si>
   <si>
     <t xml:space="preserve">Documentación y sustentación técnica</t>
@@ -612,7 +633,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="28.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="7" style="1" width="5.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="7" style="1" width="21.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="13.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="35.76"/>
   </cols>
@@ -637,7 +658,7 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="26.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1083,8 +1104,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="26.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="35.76"/>
@@ -1105,7 +1125,7 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="26.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -3092,149 +3112,149 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>20</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -3244,7 +3264,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
@@ -3255,7 +3275,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>0.7</v>
@@ -3266,7 +3286,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>0.4</v>
@@ -3277,7 +3297,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>0</v>
@@ -3310,7 +3330,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3319,7 +3339,7 @@
     </row>
     <row r="3" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -3328,7 +3348,7 @@
     </row>
     <row r="4" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -3337,7 +3357,7 @@
     </row>
     <row r="5" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -3346,7 +3366,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -3355,7 +3375,7 @@
     </row>
     <row r="7" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -3364,7 +3384,7 @@
     </row>
     <row r="8" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -3373,7 +3393,7 @@
     </row>
     <row r="9" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -3382,7 +3402,7 @@
     </row>
     <row r="10" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -3391,7 +3411,7 @@
     </row>
     <row r="11" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -3400,7 +3420,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>

</xml_diff>